<commit_message>
Fold modules 7, 8 and 21 into the QA results and regenerate
Three executed modules had never reached the overlay: client users,
PSA connections, and the public site. The scope line still said they
were session-bound and unattempted, so 30 cases carried a stamp in the
conversation and "Not run" in the document people actually read.

PUB-07 is the run's first failure and the summary page said "zero
failures", so that page is rewritten to lead with it. The Fail column
is now red - a one in that box reads as another number on the way to
the pass count when it is set in the same ink as the rest.

PUB-05 is recorded as a pass rather than the partial it was: the
truncation it found is fixed and verified in production.

Counts: 71 pass, 3 partial, 61 blocked, 8 N/A, 1 fail, 94 not run.
The 71 corrects a running total I had carried one high through module 8;
these come from the recorded per-case statuses rather than a tally kept
by hand.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/desk-portal-test-cases.xlsx
+++ b/docs/qa/desk-portal-test-cases.xlsx
@@ -3746,12 +3746,24 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr"/>
-      <c r="I60" s="5" t="inlineStr"/>
-      <c r="J60" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Needs a client session.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3786,12 +3798,24 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" s="5" t="inlineStr"/>
-      <c r="J61" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Needs an admin session. Worth noting for whoever runs it: the one client user has a null ExternalContactId, so he was invited by hand and the contact-import path has never been exercised here.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3826,12 +3850,24 @@
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr"/>
-      <c r="I62" s="5" t="inlineStr"/>
-      <c r="J62" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Needs a client session.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3866,12 +3902,24 @@
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" s="5" t="inlineStr"/>
-      <c r="J63" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>Needs a client session.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3906,12 +3954,24 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="inlineStr"/>
-      <c r="I64" s="5" t="inlineStr"/>
-      <c r="J64" s="4" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>All 355 notes carry AuthoredByClient = false - 17 portal-authored, 338 imported. That is the shape of the PR #66 bug, but it is not a regression: both connectors populate the flag and the heal loop rewrites it on every sync, of which many ran. No client has ever written a note in either PSA, so the mechanism is verified and the rendering is not - two different claims.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3946,12 +4006,24 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" s="5" t="inlineStr"/>
-      <c r="J65" s="4" t="inlineStr"/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>Zero section grants exist, so there is nothing to delegate.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3986,12 +4058,24 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H66" s="4" t="inlineStr"/>
-      <c r="I66" s="5" t="inlineStr"/>
-      <c r="J66" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Needs a client session. Last-admin protection is unit-tested.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4026,12 +4110,24 @@
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr"/>
-      <c r="I67" s="5" t="inlineStr"/>
-      <c r="J67" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>Needs a client session.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4066,12 +4162,24 @@
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr"/>
-      <c r="I68" s="5" t="inlineStr"/>
-      <c r="J68" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>The connection row holds a 32-character opaque id; the material lives in secret_blobs."Ciphertext" as bytea in a separate table. Structural, which is what the case asks - an attempt to measure how printable the ciphertext was returned 257% and meant nothing, because encode(escape) expands bytes.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4106,12 +4214,24 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" s="5" t="inlineStr"/>
-      <c r="J69" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>Needs a session. Read-only and safe to run - one call to the PSA.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4146,12 +4266,24 @@
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr"/>
-      <c r="I70" s="5" t="inlineStr"/>
-      <c r="J70" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>Needs credentials typed into a form, which is the tester's to do and not the agent's. Merge-not-clobber is unit-tested.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4186,12 +4318,24 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" s="5" t="inlineStr"/>
-      <c r="J71" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>Needs a session. Display only, safe.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4226,12 +4370,24 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H72" s="4" t="inlineStr"/>
-      <c r="I72" s="5" t="inlineStr"/>
-      <c r="J72" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>Needs a session AND stops a live integration syncing. Reversible in seconds, but it is a deliberate outage on production - staging is the honest place for it.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4266,12 +4422,24 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr"/>
-      <c r="I73" s="5" t="inlineStr"/>
-      <c r="J73" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>Needs a session. Read-only against the PSA, safe.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4306,12 +4474,24 @@
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H74" s="4" t="inlineStr"/>
-      <c r="I74" s="5" t="inlineStr"/>
-      <c r="J74" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>Map() filters o.IsActive before options reach the mapping UI.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4346,12 +4526,24 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr"/>
-      <c r="I75" s="5" t="inlineStr"/>
-      <c r="J75" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>Options carry Value and SyncValue, held by certification tests on both providers.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4386,12 +4578,24 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H76" s="4" t="inlineStr"/>
-      <c r="I76" s="5" t="inlineStr"/>
-      <c r="J76" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>Rests on the An_import_filter_restricted_to_one_company_excludes_the_others test written this run - production filters are empty, so no live data proves it. The test exists because the fake used to match everything.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4426,12 +4630,24 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr"/>
-      <c r="I77" s="5" t="inlineStr"/>
-      <c r="J77" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>The one to avoid on production: turning the toggle off and re-syncing could reconcile away the 113 already-imported closed Autotask tickets, and recovering them means another full re-sync. Real data movement to prove a toggle.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4466,12 +4682,24 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="inlineStr"/>
-      <c r="I78" s="5" t="inlineStr"/>
-      <c r="J78" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Needs a session. Creates no time entry, so safe to run.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4506,12 +4734,24 @@
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr"/>
-      <c r="I79" s="5" t="inlineStr"/>
-      <c r="J79" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>Needs a session, but arguably already covered: the button calls the same ConnectionSyncRunner invoked a dozen times this run by resetting the watermark. Only the HTTP entry point is untested.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4546,12 +4786,24 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="inlineStr"/>
-      <c r="I80" s="5" t="inlineStr"/>
-      <c r="J80" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Both connections healthy, enabled, synced within the minute, no error.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4586,12 +4838,24 @@
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H81" s="4" t="inlineStr"/>
-      <c r="I81" s="5" t="inlineStr"/>
-      <c r="J81" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>A failed run sets Status = Degraded and LastError, cleared on success. Corroborated by the Autotask 405 incident this run, which exercised the path for real - LastError reads empty now precisely because the next success cleared it.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -10466,12 +10730,24 @@
       </c>
       <c r="G216" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H216" s="4" t="inlineStr"/>
-      <c r="I216" s="5" t="inlineStr"/>
-      <c r="J216" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H216" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I216" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J216" s="4" t="inlineStr">
+        <is>
+          <t>All 17 public pages return 200 with real content, not a shell.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -10506,12 +10782,24 @@
       </c>
       <c r="G217" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H217" s="4" t="inlineStr"/>
-      <c r="I217" s="5" t="inlineStr"/>
-      <c r="J217" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H217" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I217" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J217" s="4" t="inlineStr">
+        <is>
+          <t>Stored with Kind = 0. The test rows were deleted afterwards; the one genuine enquiry on production was left alone.</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -10546,12 +10834,24 @@
       </c>
       <c r="G218" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H218" s="4" t="inlineStr"/>
-      <c r="I218" s="5" t="inlineStr"/>
-      <c r="J218" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H218" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I218" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J218" s="4" t="inlineStr">
+        <is>
+          <t>Stored with Kind = 1, carrying the preferred time as the visitor worded it.</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -10586,12 +10886,24 @@
       </c>
       <c r="G219" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H219" s="4" t="inlineStr"/>
-      <c r="I219" s="5" t="inlineStr"/>
-      <c r="J219" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H219" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I219" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J219" s="4" t="inlineStr">
+        <is>
+          <t>A filled honeypot answers 202 and stores nothing - confirmed by row count.</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -10626,12 +10938,24 @@
       </c>
       <c r="G220" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H220" s="4" t="inlineStr"/>
-      <c r="I220" s="5" t="inlineStr"/>
-      <c r="J220" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H220" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I220" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J220" s="4" t="inlineStr">
+        <is>
+          <t>A defect this run, now fixed and verified in production. A 60,000-character message used to return 202 and store exactly 4,000: the sender was thanked and never told, and staff read a message ending mid-sentence with nothing to mark the cut. Every visitor-typed field is now refused when oversized, naming the field and the limit, and nothing is written on a refusal. Live: 60,000 and 4,001 both 400, a normal message 202, no truncated rows. SourcePage is still clipped on purpose - the site fills it in, and a lead should not be lost to the length of our own URL.</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -10666,12 +10990,24 @@
       </c>
       <c r="G221" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H221" s="4" t="inlineStr"/>
-      <c r="I221" s="5" t="inlineStr"/>
-      <c r="J221" s="4" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H221" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I221" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J221" s="4" t="inlineStr">
+        <is>
+          <t>Needs an admin session to move an enquiry through its statuses.</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -10706,12 +11042,24 @@
       </c>
       <c r="G222" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H222" s="4" t="inlineStr"/>
-      <c r="I222" s="5" t="inlineStr"/>
-      <c r="J222" s="4" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H222" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I222" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J222" s="4" t="inlineStr">
+        <is>
+          <t>Twelve unfilled placeholders are live and visible: seven on /privacy (registered address, hosting provider, hosting region, and four retention periods reading "e.g. 24 months" and the like) and five on /terms (two notice periods, the liability cap "e.g. the fees paid in the preceding 12 months", and governing law twice as "your jurisdiction"). A scan for placeholder MARKERS - TBD, TODO, lorem ipsum - finds nothing, because the slots hold ordinary English inside &lt;mark&gt; elements; only grepping "&lt;Fill" in the page sources revealed them. Needs the owner's real values.</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -10746,12 +11094,24 @@
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="H223" s="4" t="inlineStr"/>
-      <c r="I223" s="5" t="inlineStr"/>
-      <c r="J223" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H223" s="4" t="inlineStr">
+        <is>
+          <t>Claude (agent), unattended - no interactive session available</t>
+        </is>
+      </c>
+      <c r="I223" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05 / 06 / 07</t>
+        </is>
+      </c>
+      <c r="J223" s="4" t="inlineStr">
+        <is>
+          <t>Zero cookies are set on any public page, so no banner is owed. The session cookies begin at sign-in and are strictly necessary.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -11581,7 +11941,7 @@
       </c>
       <c r="J239" s="4" t="inlineStr">
         <is>
-          <t>540 unit tests green; five defects this run were each hidden at least once by a fake more permissive than the real API, and each fake was tightened.</t>
+          <t>549 unit tests green; five defects this run were each hidden at least once by a fake more permissive than the real API, and each fake was tightened.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill the registered address, closing PUB-07
The last of the twelve. F-88, Phase 8B, Industrial Area, Mohali, Punjab
160055, India, supplied by the owner - it is a fact about the filed entity
and was never ours to infer from an office location.

Zero placeholder spans remain on either page, so the Fill component is now
unused by both; its imports go with it. The component itself stays, because
the next legal document will want the same visible marker.

PUB-07 moves from Fail to Pass and the run has no failures left. Its result
keeps the story rather than just the verdict: the placeholders were invisible
to a marker scan because they held ordinary English, and the retention slots
turned out to be promises the software could not keep.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/desk-portal-test-cases.xlsx
+++ b/docs/qa/desk-portal-test-cases.xlsx
@@ -11106,7 +11106,7 @@
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H223" s="4" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="J223" s="4" t="inlineStr">
         <is>
-          <t>Twelve unfilled placeholders are live and visible: seven on /privacy (registered address, hosting provider, hosting region, and four retention periods reading "e.g. 24 months" and the like) and five on /terms (two notice periods, the liability cap "e.g. the fees paid in the preceding 12 months", and governing law twice as "your jurisdiction"). A scan for placeholder MARKERS - TBD, TODO, lorem ipsum - finds nothing, because the slots hold ordinary English inside &lt;mark&gt; elements; only grepping "&lt;Fill" in the page sources revealed them. Needs the owner's real values.</t>
+          <t>Failed when first run: twelve unfilled placeholders were live and visible - seven on /privacy and five on /terms, including retention periods reading "e.g. 24 months" and governing law as "your jurisdiction". A scan for placeholder MARKERS (TBD, TODO, lorem ipsum) found nothing, because the slots held ordinary English inside &lt;mark&gt; elements; only grepping "&lt;Fill" in the page sources revealed them. All twelve are now filled and zero &lt;mark&gt; spans remain on either live page. The retention ones were not blanks but promises: nothing deletes enquiries or audit records and logs rotate at 14 days, so the policy states what the system actually does rather than periods no code enforces. Hosting is named from the host's own network (Hostinger, United States) - the owner should confirm the region in their panel, as it decides whether EU data is being transferred.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill the registered address, closing PUB-07 (#155)
The last of the twelve. F-88, Phase 8B, Industrial Area, Mohali, Punjab
160055, India, supplied by the owner - it is a fact about the filed entity
and was never ours to infer from an office location.

Zero placeholder spans remain on either page, so the Fill component is now
unused by both; its imports go with it. The component itself stays, because
the next legal document will want the same visible marker.

PUB-07 moves from Fail to Pass and the run has no failures left. Its result
keeps the story rather than just the verdict: the placeholders were invisible
to a marker scan because they held ordinary English, and the retention slots
turned out to be promises the software could not keep.

Co-authored-by: Desk Portal <proapps@techpio.com>
Co-authored-by: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/desk-portal-test-cases.xlsx
+++ b/docs/qa/desk-portal-test-cases.xlsx
@@ -11106,7 +11106,7 @@
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H223" s="4" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="J223" s="4" t="inlineStr">
         <is>
-          <t>Twelve unfilled placeholders are live and visible: seven on /privacy (registered address, hosting provider, hosting region, and four retention periods reading "e.g. 24 months" and the like) and five on /terms (two notice periods, the liability cap "e.g. the fees paid in the preceding 12 months", and governing law twice as "your jurisdiction"). A scan for placeholder MARKERS - TBD, TODO, lorem ipsum - finds nothing, because the slots hold ordinary English inside &lt;mark&gt; elements; only grepping "&lt;Fill" in the page sources revealed them. Needs the owner's real values.</t>
+          <t>Failed when first run: twelve unfilled placeholders were live and visible - seven on /privacy and five on /terms, including retention periods reading "e.g. 24 months" and governing law as "your jurisdiction". A scan for placeholder MARKERS (TBD, TODO, lorem ipsum) found nothing, because the slots held ordinary English inside &lt;mark&gt; elements; only grepping "&lt;Fill" in the page sources revealed them. All twelve are now filled and zero &lt;mark&gt; spans remain on either live page. The retention ones were not blanks but promises: nothing deletes enquiries or audit records and logs rotate at 14 days, so the policy states what the system actually does rather than periods no code enforces. Hosting is named from the host's own network (Hostinger, United States) - the owner should confirm the region in their panel, as it decides whether EU data is being transferred.</t>
         </is>
       </c>
     </row>

</xml_diff>